<commit_message>
Login tc 3 & 4 and modifications to relative classes
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,20 +3,34 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="InvalidLoginCredentials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LoginCredentials" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LogoutData" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="InvalidLoginCredentials" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FDValidation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>IncorrectPassword</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>emailSentSuccessMsg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both sms and email sending are success</t>
+  </si>
+  <si>
+    <t>popupText</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are you sure you want to logout?</t>
+  </si>
+  <si>
+    <t>incorrectPassword</t>
   </si>
   <si>
     <t>errorMessage</t>
@@ -28,22 +42,34 @@
     <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS</t>
   </si>
   <si>
-    <t>userName</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t>expectedMsg</t>
-  </si>
-  <si>
-    <t>botuser</t>
-  </si>
-  <si>
-    <t>Hoax@1234</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email sent successfully to the registered email address</t>
+    <t>fDAccountNumber</t>
+  </si>
+  <si>
+    <t>currencyAndAvailableBalance</t>
+  </si>
+  <si>
+    <t>maturityAmount</t>
+  </si>
+  <si>
+    <t>maturityDate</t>
+  </si>
+  <si>
+    <t>interestRate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2061 5750 3998</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 3,000,000.00</t>
+  </si>
+  <si>
+    <t>3,000,000.00</t>
+  </si>
+  <si>
+    <t>08/06/2025</t>
+  </si>
+  <si>
+    <t>8.5%</t>
   </si>
 </sst>
 </file>
@@ -59,6 +85,7 @@
     </font>
     <font>
       <sz val="10.000000"/>
+      <color rgb="FF6AAB73"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -82,11 +109,12 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -595,24 +623,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.421875"/>
-    <col customWidth="1" min="2" max="2" width="27.28125"/>
+    <col customWidth="1" min="1" max="1" width="21.28125"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -626,27 +647,108 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="25.8515625"/>
+  </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="21.421875"/>
+    <col customWidth="1" min="2" max="2" width="27.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="18.00390625"/>
+    <col customWidth="1" min="2" max="2" width="27.140625"/>
+    <col customWidth="1" min="3" max="3" width="16.28125"/>
+    <col customWidth="1" min="4" max="5" width="16.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
       <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added dashboard tc with few modifications to base page and common utils
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,20 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="InvalidLoginCredentials" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="LogoutData" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FDValidation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DashboardSavingsValidationData" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DashboardFDValidation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DashboardRVTTransferValidOLD" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>userName</t>
   </si>
@@ -54,12 +56,27 @@
     <t xml:space="preserve">Are you sure you want to logout?</t>
   </si>
   <si>
+    <t>savingsAccountNumber</t>
+  </si>
+  <si>
+    <t>currencyAndAvailableBalance</t>
+  </si>
+  <si>
+    <t>productName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1001 5102 6073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 880.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE S SAVINGS -PERSONAL</t>
+  </si>
+  <si>
     <t>fDAccountNumber</t>
   </si>
   <si>
-    <t>currencyAndAvailableBalance</t>
-  </si>
-  <si>
     <t>maturityAmount</t>
   </si>
   <si>
@@ -82,6 +99,24 @@
   </si>
   <si>
     <t>8.5%</t>
+  </si>
+  <si>
+    <t>accountName</t>
+  </si>
+  <si>
+    <t>currencyAndAmount</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 350.00;LKR 300.00;LKR 200.00;LKR 1,776.45;LKR 330.00;LKR 153.00;LKR 1,000.00;LKR 255.00;LKR 250.00;LKR 500.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025</t>
   </si>
 </sst>
 </file>
@@ -121,15 +156,19 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -638,6 +677,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="2" max="2" width="30.8515625"/>
     <col customWidth="1" min="3" max="3" width="21.28125"/>
   </cols>
   <sheetData>
@@ -762,6 +802,45 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="29.421875"/>
+    <col customWidth="1" min="2" max="2" width="26.140625"/>
+    <col customWidth="1" min="3" max="3" width="20.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
     <col customWidth="1" min="1" max="1" width="18.00390625"/>
     <col customWidth="1" min="2" max="2" width="27.140625"/>
     <col customWidth="1" min="3" max="3" width="16.28125"/>
@@ -769,37 +848,76 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>16</v>
+      <c r="C1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="48.00390625"/>
+    <col customWidth="1" min="2" max="2" width="55.7109375"/>
+    <col customWidth="1" min="3" max="3" width="48.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" ht="67.5" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added dashboard tc with some methods in base pge and common utils
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,13 +12,14 @@
     <sheet name="DashboardSavingsValidationData" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DashboardFDValidation" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DashboardRVTTransferValidOLD" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DashboardLoanValidation" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>userName</t>
   </si>
@@ -117,13 +118,37 @@
   </si>
   <si>
     <t xml:space="preserve">Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025;Feb 24, 2025</t>
+  </si>
+  <si>
+    <t>loanAccountNumber</t>
+  </si>
+  <si>
+    <t>loanAmt</t>
+  </si>
+  <si>
+    <t>outstanding</t>
+  </si>
+  <si>
+    <t>loanPeriod</t>
+  </si>
+  <si>
+    <t>300164007642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 5,000.00</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>8.98%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -134,6 +159,11 @@
       <sz val="10.000000"/>
       <color rgb="FF6AAB73"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9.000000"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
     </font>
   </fonts>
   <fills count="2">
@@ -156,12 +186,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -169,6 +198,10 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,7 +855,7 @@
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -848,19 +881,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>21</v>
       </c>
     </row>
@@ -899,25 +932,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="2" ht="67.5" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="34.421875"/>
+    <col customWidth="1" min="2" max="2" width="21.00390625"/>
+    <col customWidth="1" min="3" max="4" width="17.421875"/>
+    <col customWidth="1" min="5" max="5" width="26.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added dashboard regression tc with some methods in base pge and common utils
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="6"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,13 +13,14 @@
     <sheet name="DashboardFDValidation" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DashboardRVTTransferValidOLD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="DashboardLoanValidation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DashboardRVTPaymentPopup" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>userName</t>
   </si>
@@ -45,6 +46,12 @@
     <t>errorMessage</t>
   </si>
   <si>
+    <t>ceftissue</t>
+  </si>
+  <si>
+    <t>Abcd@1234</t>
+  </si>
+  <si>
     <t>tgeffrf</t>
   </si>
   <si>
@@ -69,7 +76,7 @@
     <t xml:space="preserve">1001 5102 6073</t>
   </si>
   <si>
-    <t xml:space="preserve">LKR 880.00</t>
+    <t xml:space="preserve">LKR 9,880.00</t>
   </si>
   <si>
     <t xml:space="preserve">DOUBLE S SAVINGS -PERSONAL</t>
@@ -142,6 +149,12 @@
   </si>
   <si>
     <t>8.98%</t>
+  </si>
+  <si>
+    <t>toAccount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceylon Electricity Board</t>
   </si>
 </sst>
 </file>
@@ -186,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -201,7 +214,6 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -710,6 +722,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="20.57421875"/>
     <col customWidth="1" min="2" max="2" width="30.8515625"/>
     <col customWidth="1" min="3" max="3" width="21.28125"/>
   </cols>
@@ -729,10 +742,10 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -748,6 +761,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="2" max="2" width="20.421875"/>
     <col customWidth="1" min="3" max="3" width="21.421875"/>
     <col customWidth="1" min="4" max="4" width="27.28125"/>
   </cols>
@@ -768,16 +782,16 @@
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -806,7 +820,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" ht="14.25">
@@ -820,7 +834,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -842,24 +856,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -882,36 +896,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -933,24 +947,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" ht="67.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +977,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="34.421875"/>
     <col customWidth="1" min="2" max="2" width="21.00390625"/>
@@ -973,36 +987,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>40</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added additional dashboard regression tc with some methods in base pge and common utils
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,24 +3,26 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="InvalidLoginCredentials" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LogoutData" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DashboardSavingsValidationData" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DashboardFDValidation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DashboardRVTTransferValidOLD" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DashboardLoanValidation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DashboardRVTPaymentPopup" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="LoginDataAlternateOne" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="InvalidLoginCredentials" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LogoutData" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DashboardSavingsValidationData" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DashboardFDValidation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DashboardRVTTransferValidOLD" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DashboardLoanValidation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DashboardRVTPaymentPopup" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DashboardAccountPortfolio" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>userName</t>
   </si>
@@ -40,6 +42,12 @@
     <t xml:space="preserve">Both sms and email sending are success</t>
   </si>
   <si>
+    <t>settlement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMS sent successfully to the registered mobile number</t>
+  </si>
+  <si>
     <t>incorrectPassword</t>
   </si>
   <si>
@@ -155,6 +163,18 @@
   </si>
   <si>
     <t xml:space="preserve">Ceylon Electricity Board</t>
+  </si>
+  <si>
+    <t>imgLocation</t>
+  </si>
+  <si>
+    <t>threshold</t>
+  </si>
+  <si>
+    <t>src/test/resources/IMAGE-VERIFICATIONS/AccountPortfolioSettlement.png</t>
+  </si>
+  <si>
+    <t>80</t>
   </si>
 </sst>
 </file>
@@ -199,8 +219,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -214,6 +237,7 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -757,7 +781,84 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="12.8515625"/>
+    <col customWidth="1" min="2" max="2" width="12.28125"/>
+    <col customWidth="1" min="3" max="3" width="14.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="31.00390625"/>
+    <col customWidth="1" min="3" max="3" width="45.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -774,24 +875,24 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -820,7 +921,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" ht="14.25">
@@ -834,7 +935,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -845,7 +946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -856,24 +957,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -884,7 +985,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -895,37 +996,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="B1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>23</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>28</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -936,7 +1037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -946,25 +1047,25 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="B1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="2" ht="67.5" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>34</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -975,7 +1076,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -986,37 +1087,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>23</v>
+      <c r="C1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="A2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>42</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1027,18 +1128,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added transfers and biller template page and modifications to util and base pages
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,26 +3,30 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="9"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LoginDataAlternateOne" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="InvalidLoginCredentials" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="LogoutData" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DashboardSavingsValidationData" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DashboardFDValidation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DashboardRVTTransferValidOLD" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DashboardLoanValidation" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="DashboardRVTPaymentPopup" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DashboardAccountPortfolio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="InvalidResetUser" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LockedUserReset" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="InvalidSecurityAnswer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LoginDataAlternateOne" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LockedCredential" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="InvalidLoginCredentials" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LogoutData" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DashboardSavingsValidationData" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DashboardFDValidation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DashboardRVTTransferValidOLD" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DashboardLoanValidation" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DashboardRVTPaymentPopup" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DashboardAccountPortfolio" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>userName</t>
   </si>
@@ -42,18 +46,39 @@
     <t xml:space="preserve">Both sms and email sending are success</t>
   </si>
   <si>
+    <t>incorrectUser</t>
+  </si>
+  <si>
+    <t>errorMessage</t>
+  </si>
+  <si>
+    <t>uioirhjkhj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incorrect user ID . Please recheck and try again.</t>
+  </si>
+  <si>
+    <t>deluxe86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your user ID is locked. Please contact the customer care center 011 2 30 30 50 or visit the nearest branch.</t>
+  </si>
+  <si>
+    <t>mvijtha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incorrect answer. Please recheck and try again</t>
+  </si>
+  <si>
     <t>settlement</t>
   </si>
   <si>
-    <t xml:space="preserve">SMS sent successfully to the registered mobile number</t>
+    <t xml:space="preserve">YOUR ACCOUNT IS LOCKED. PLEASE CONTACT CALL CENTRE FOR FURTHER ASSISTANCE.</t>
   </si>
   <si>
     <t>incorrectPassword</t>
   </si>
   <si>
-    <t>errorMessage</t>
-  </si>
-  <si>
     <t>ceftissue</t>
   </si>
   <si>
@@ -84,7 +109,7 @@
     <t xml:space="preserve">1001 5102 6073</t>
   </si>
   <si>
-    <t xml:space="preserve">LKR 9,880.00</t>
+    <t xml:space="preserve">LKR 8,730.00</t>
   </si>
   <si>
     <t xml:space="preserve">DOUBLE S SAVINGS -PERSONAL</t>
@@ -174,7 +199,7 @@
     <t>src/test/resources/IMAGE-VERIFICATIONS/AccountPortfolioSettlement.png</t>
   </si>
   <si>
-    <t>80</t>
+    <t>200</t>
   </si>
 </sst>
 </file>
@@ -219,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -237,7 +262,6 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -783,7 +807,172 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="18.00390625"/>
+    <col customWidth="1" min="2" max="2" width="27.140625"/>
+    <col customWidth="1" min="3" max="3" width="16.28125"/>
+    <col customWidth="1" min="4" max="5" width="16.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="48.00390625"/>
+    <col customWidth="1" min="2" max="2" width="55.7109375"/>
+    <col customWidth="1" min="3" max="3" width="48.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" ht="67.5" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="34.421875"/>
+    <col customWidth="1" min="2" max="2" width="21.00390625"/>
+    <col customWidth="1" min="3" max="4" width="17.421875"/>
+    <col customWidth="1" min="5" max="5" width="26.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="12.8515625"/>
     <col customWidth="1" min="2" max="2" width="12.28125"/>
@@ -792,24 +981,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>50</v>
+        <v>14</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -822,8 +1011,105 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="20.00390625"/>
+    <col customWidth="1" min="2" max="2" width="43.421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="20.7109375"/>
+    <col customWidth="1" min="2" max="2" width="53.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="38.7109375"/>
+    <col customWidth="1" min="2" max="2" width="52.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="19.421875"/>
     <col customWidth="1" min="2" max="2" width="31.00390625"/>
     <col customWidth="1" min="3" max="3" width="45.28125"/>
   </cols>
@@ -839,15 +1125,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
+    <row r="2" ht="14.25">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -858,7 +1144,45 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="17.7109375"/>
+    <col customWidth="1" min="3" max="3" width="29.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -875,24 +1199,24 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -903,7 +1227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -921,7 +1245,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="14.25">
@@ -935,7 +1259,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -946,7 +1270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -957,189 +1281,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="18.00390625"/>
-    <col customWidth="1" min="2" max="2" width="27.140625"/>
-    <col customWidth="1" min="3" max="3" width="16.28125"/>
-    <col customWidth="1" min="4" max="5" width="16.8515625"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="48.00390625"/>
-    <col customWidth="1" min="2" max="2" width="55.7109375"/>
-    <col customWidth="1" min="3" max="3" width="48.28125"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" ht="67.5" customHeight="1">
-      <c r="A2" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="34.421875"/>
-    <col customWidth="1" min="2" max="2" width="21.00390625"/>
-    <col customWidth="1" min="3" max="4" width="17.421875"/>
-    <col customWidth="1" min="5" max="5" width="26.140625"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <sheetData>
-    <row r="1" ht="14.25">
-      <c r="A1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25">
-      <c r="A2" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified Billers and transfers and general enhancements to other pages
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,30 +3,34 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="InvalidResetUser" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LockedUserReset" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="InvalidSecurityAnswer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="LoginDataAlternateOne" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="LockedCredential" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="InvalidLoginCredentials" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="LogoutData" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="DashboardSavingsValidationData" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DashboardFDValidation" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="DashboardRVTTransferValidOLD" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="DashboardLoanValidation" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DashboardRVTPaymentPopup" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="DashboardAccountPortfolio" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="LoginDataAlternateOne" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LoginDataAlternateTwo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LoginDataAlternateThree" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BillPayments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BillPayments2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="InvalidResetUser" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LockedUserReset" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="InvalidSecurityAnswer" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="LockedCredential" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="InvalidLoginCredentials" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="LogoutData" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DashboardSavingsValidationData" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DashboardFDValidation" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DashboardRVTTransferValidOLD" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DashboardLoanValidation" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="DashboardRVTPaymentPopup" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="DashboardAccountPortfolio" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
   <si>
     <t>userName</t>
   </si>
@@ -43,9 +47,453 @@
     <t>Hoax@1234</t>
   </si>
   <si>
+    <t xml:space="preserve">SMS sent successfully to the registered mobile num</t>
+  </si>
+  <si>
+    <t>settlement</t>
+  </si>
+  <si>
+    <t>mvijtha</t>
+  </si>
+  <si>
+    <t>maheshmahendra</t>
+  </si>
+  <si>
     <t xml:space="preserve">Both sms and email sending are success</t>
   </si>
   <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>billerName</t>
+  </si>
+  <si>
+    <t>paymentUsing</t>
+  </si>
+  <si>
+    <t>transferMode</t>
+  </si>
+  <si>
+    <t>fromAccount</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>mobileNo</t>
+  </si>
+  <si>
+    <t>accountNumber</t>
+  </si>
+  <si>
+    <t>errorMsgOne</t>
+  </si>
+  <si>
+    <t>errorMsgTwo</t>
+  </si>
+  <si>
+    <t>errorMsgThree</t>
+  </si>
+  <si>
+    <t>errorMsgFour</t>
+  </si>
+  <si>
+    <t>errorMsgFive</t>
+  </si>
+  <si>
+    <t>errorMsgSix</t>
+  </si>
+  <si>
+    <t>nicNo</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>policyNumber</t>
+  </si>
+  <si>
+    <t>admissionNumber</t>
+  </si>
+  <si>
+    <t>classID</t>
+  </si>
+  <si>
+    <t>purpose</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>referenceOrReservationNo</t>
+  </si>
+  <si>
+    <t>employeeID</t>
+  </si>
+  <si>
+    <t>branch</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Telephone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog Mobile</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time Transaction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1022 5214 6593</t>
+  </si>
+  <si>
+    <t>0775446565</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your GSM Phone Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobitel Pvt Ltd</t>
+  </si>
+  <si>
+    <t>0718642894</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobitel Phone Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIRTEL [Prepaid &amp; Postpaid]</t>
+  </si>
+  <si>
+    <t>0758642894</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airtel Phone Number is required</t>
+  </si>
+  <si>
+    <t>HUTCH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sri Lanka Telecom - New Invoice Numbers(14 Digits)</t>
+  </si>
+  <si>
+    <t>0114245643</t>
+  </si>
+  <si>
+    <t>1587456456-4646</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice Number With (-) is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telephone Number with Area Code is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable - TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog TV</t>
+  </si>
+  <si>
+    <t>1232034656</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account No is required</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sri Lanka Insurance - Life Renewals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy No is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of Policy Holder is required</t>
+  </si>
+  <si>
+    <t>Sampath</t>
+  </si>
+  <si>
+    <t>5432156</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Janashakthi Insurance Co. Ltd - Life</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIC Number  is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy Number is required</t>
+  </si>
+  <si>
+    <t>856546546546</t>
+  </si>
+  <si>
+    <t>88956724654641354545</t>
+  </si>
+  <si>
+    <t xml:space="preserve">School Fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Musaeus College</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student Admission Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student Name is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purpose is required</t>
+  </si>
+  <si>
+    <t>564646464446</t>
+  </si>
+  <si>
+    <t>5C</t>
+  </si>
+  <si>
+    <t>fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S. Thomas' College</t>
+  </si>
+  <si>
+    <t>5646464</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internet Service Providers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog Broadband</t>
+  </si>
+  <si>
+    <t>0745465465</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone No is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sri Lanka Telecom - 4G</t>
+  </si>
+  <si>
+    <t>0118565464</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4G Telephone Number with Area Code is required</t>
+  </si>
+  <si>
+    <t>Hospitals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durdans Hospital</t>
+  </si>
+  <si>
+    <t>556468</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient's Reference Number BHT is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name Of The Patient is required</t>
+  </si>
+  <si>
+    <t>Sumith</t>
+  </si>
+  <si>
+    <t>CEB</t>
+  </si>
+  <si>
+    <t>2893549217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electricity Bill Account No is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financial Institutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinhaputhra Finance PLC</t>
+  </si>
+  <si>
+    <t>411546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Savings Account No. is required</t>
+  </si>
+  <si>
+    <t>Leasing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assetline Leasing Company Ltd.</t>
+  </si>
+  <si>
+    <t>0774833496</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Bank Reference No is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telephone No (10 digits) is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle No / NIC No is required</t>
+  </si>
+  <si>
+    <t>925875684465</t>
+  </si>
+  <si>
+    <t>58908908</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Srilanka Institute Of Information Technology SLIIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student Registration Number / Student NIC Number is required</t>
+  </si>
+  <si>
+    <t>FEE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National School Of Business Management Ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIC is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student Registration Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study Year is required</t>
+  </si>
+  <si>
+    <t>Donald</t>
+  </si>
+  <si>
+    <t>669588848221254</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile Money</t>
+  </si>
+  <si>
+    <t>eZCash</t>
+  </si>
+  <si>
+    <t>774546546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile Number (Without "0") is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobitel mCash</t>
+  </si>
+  <si>
+    <t>0714546546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile Wallet Number is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real Estate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Lands (Pvt) Ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Code is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservation Number is required</t>
+  </si>
+  <si>
+    <t>5564646465</t>
+  </si>
+  <si>
+    <t>4765468654</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clubs &amp; Societies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAACHA - Photography Club Of Sampath Bank</t>
+  </si>
+  <si>
+    <t>0775646546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calling Name is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employee ID is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email address is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact No is required</t>
+  </si>
+  <si>
+    <t>sunil</t>
+  </si>
+  <si>
+    <t>Colombo</t>
+  </si>
+  <si>
+    <t>sunilt@gmail.com</t>
+  </si>
+  <si>
+    <t>LECO</t>
+  </si>
+  <si>
+    <t>0306306902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing Month (YYYYMM) is required</t>
+  </si>
+  <si>
+    <t>202405</t>
+  </si>
+  <si>
+    <t>NWSDB</t>
+  </si>
+  <si>
+    <t>125531351351</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only the first 12 numbers of Water Bill Account Nu is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year/Month of the Bill (YYYYMM) is required</t>
+  </si>
+  <si>
     <t>incorrectUser</t>
   </si>
   <si>
@@ -64,15 +512,9 @@
     <t xml:space="preserve">Your user ID is locked. Please contact the customer care center 011 2 30 30 50 or visit the nearest branch.</t>
   </si>
   <si>
-    <t>mvijtha</t>
-  </si>
-  <si>
     <t xml:space="preserve">Incorrect answer. Please recheck and try again</t>
   </si>
   <si>
-    <t>settlement</t>
-  </si>
-  <si>
     <t xml:space="preserve">YOUR ACCOUNT IS LOCKED. PLEASE CONTACT CALL CENTRE FOR FURTHER ASSISTANCE.</t>
   </si>
   <si>
@@ -109,7 +551,7 @@
     <t xml:space="preserve">1001 5102 6073</t>
   </si>
   <si>
-    <t xml:space="preserve">LKR 8,730.00</t>
+    <t xml:space="preserve">LKR 8,530.00</t>
   </si>
   <si>
     <t xml:space="preserve">DOUBLE S SAVINGS -PERSONAL</t>
@@ -146,9 +588,6 @@
   </si>
   <si>
     <t>currencyAndAmount</t>
-  </si>
-  <si>
-    <t>date</t>
   </si>
   <si>
     <t xml:space="preserve">Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account,Own Account</t>
@@ -206,7 +645,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -214,14 +653,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9.000000"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="10.000000"/>
       <color rgb="FF6AAB73"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.000000"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Courier New"/>
     </font>
   </fonts>
   <fills count="2">
@@ -244,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="26">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -252,14 +697,58 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -793,7 +1282,7 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -809,44 +1298,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.00390625"/>
-    <col customWidth="1" min="2" max="2" width="27.140625"/>
-    <col customWidth="1" min="3" max="3" width="16.28125"/>
-    <col customWidth="1" min="4" max="5" width="16.8515625"/>
+    <col customWidth="1" min="2" max="2" width="17.7109375"/>
+    <col customWidth="1" min="3" max="3" width="29.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>32</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>37</v>
+      <c r="A2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -861,31 +1336,37 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="48.00390625"/>
-    <col customWidth="1" min="2" max="2" width="55.7109375"/>
-    <col customWidth="1" min="3" max="3" width="48.28125"/>
+    <col customWidth="1" min="2" max="2" width="20.421875"/>
+    <col customWidth="1" min="3" max="3" width="21.421875"/>
+    <col customWidth="1" min="4" max="4" width="27.28125"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" ht="67.5" customHeight="1">
-      <c r="A2" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>43</v>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -900,44 +1381,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="34.421875"/>
-    <col customWidth="1" min="2" max="2" width="21.00390625"/>
-    <col customWidth="1" min="3" max="4" width="17.421875"/>
-    <col customWidth="1" min="5" max="5" width="26.140625"/>
+    <col customWidth="1" min="3" max="3" width="25.8515625"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>51</v>
+    <row r="1" ht="14.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -951,15 +1423,32 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="29.421875"/>
+    <col customWidth="1" min="2" max="2" width="26.140625"/>
+    <col customWidth="1" min="3" max="3" width="20.57421875"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1">
       <c r="A1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25">
-      <c r="A2" t="s">
-        <v>53</v>
+        <v>169</v>
+      </c>
+      <c r="B1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -974,31 +1463,196 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.8515625"/>
+    <col customWidth="1" min="1" max="1" width="18.00390625"/>
+    <col customWidth="1" min="2" max="2" width="27.140625"/>
+    <col customWidth="1" min="3" max="3" width="16.28125"/>
+    <col customWidth="1" min="4" max="5" width="16.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="48.00390625"/>
+    <col customWidth="1" min="2" max="2" width="55.7109375"/>
+    <col customWidth="1" min="3" max="3" width="48.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" ht="67.5" customHeight="1">
+      <c r="A2" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>188</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="34.421875"/>
+    <col customWidth="1" min="2" max="2" width="21.00390625"/>
+    <col customWidth="1" min="3" max="4" width="17.421875"/>
+    <col customWidth="1" min="5" max="5" width="26.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="82.00390625"/>
     <col customWidth="1" min="2" max="2" width="12.28125"/>
     <col customWidth="1" min="3" max="3" width="14.00390625"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>54</v>
+        <v>199</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>57</v>
+        <v>6</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -1013,24 +1667,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="20.00390625"/>
-    <col customWidth="1" min="2" max="2" width="43.421875"/>
+    <col customWidth="1" min="1" max="1" width="19.421875"/>
+    <col customWidth="1" min="2" max="2" width="31.00390625"/>
+    <col customWidth="1" min="3" max="3" width="45.28125"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1045,8 +1706,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="20.7109375"/>
-    <col customWidth="1" min="2" max="2" width="53.00390625"/>
+    <col customWidth="1" min="1" max="1" width="37.00390625"/>
+    <col customWidth="1" min="4" max="4" width="47.57421875"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1054,15 +1715,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1075,10 +1742,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="38.7109375"/>
-    <col customWidth="1" min="2" max="2" width="52.00390625"/>
+    <col customWidth="1" min="1" max="1" width="15.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1086,15 +1752,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1109,34 +1781,1114 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="19.421875"/>
-    <col customWidth="1" min="2" max="2" width="31.00390625"/>
-    <col customWidth="1" min="3" max="3" width="45.28125"/>
+    <col customWidth="1" min="2" max="2" width="20.8515625"/>
+    <col customWidth="1" min="7" max="7" width="30.00390625"/>
+    <col customWidth="1" min="8" max="8" width="21.7109375"/>
+    <col customWidth="1" min="9" max="9" width="17.00390625"/>
+    <col customWidth="1" min="10" max="10" width="16.57421875"/>
+    <col customWidth="1" min="11" max="14" width="17.421875"/>
+    <col customWidth="1" min="15" max="15" width="14.8515625"/>
+    <col customWidth="1" min="17" max="17" width="23.8515625"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25">
-      <c r="A2" s="1" t="s">
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>26</v>
+      </c>
+      <c r="R1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="T1" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" ht="42.75">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="A3" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" ht="28.5">
+      <c r="A4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" ht="42.75">
+      <c r="A6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="1">
+        <v>100</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="1">
+        <v>100</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" ht="28.5">
+      <c r="A8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="1">
+        <v>100</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="P8" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q8" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" ht="28.5">
+      <c r="A9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="1">
+        <v>100</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="P9" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q9" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" ht="57">
+      <c r="A10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="1">
+        <v>100</v>
+      </c>
+      <c r="G10" s="11"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="N10" s="6"/>
+      <c r="O10" s="11"/>
+      <c r="P10" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="S10" t="s">
+        <v>78</v>
+      </c>
+      <c r="T10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" ht="33.75">
+      <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="1">
+        <v>100</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="11"/>
+      <c r="P11" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="S11" t="s">
+        <v>78</v>
+      </c>
+      <c r="T11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" ht="28.5">
+      <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="1">
+        <v>100</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="12"/>
+      <c r="I12" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="11"/>
+      <c r="P12"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12"/>
+      <c r="T12"/>
+    </row>
+    <row r="13" ht="42.75">
+      <c r="A13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="1">
+        <v>100</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="H13" t="s">
+        <v>53</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" ht="45">
+      <c r="A14" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="1">
+        <v>100</v>
+      </c>
+      <c r="G14" s="11"/>
+      <c r="H14" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="L14" s="18"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+    </row>
+    <row r="15" ht="33.75">
+      <c r="A15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="1">
+        <v>100</v>
+      </c>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="16"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
+      <c r="Y15" s="1"/>
+      <c r="Z15" s="1"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="1">
+        <v>100</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" t="s">
+        <v>101</v>
+      </c>
+      <c r="J16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" s="11" customFormat="1" ht="42.75">
+      <c r="A17" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="1">
+        <v>100</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="11"/>
+      <c r="I17" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="J17" s="6"/>
+      <c r="K17" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="1"/>
+      <c r="W17" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="X17" s="1"/>
+      <c r="Y17" s="1"/>
+      <c r="Z17" s="1"/>
+    </row>
+    <row r="18" ht="56.25">
+      <c r="A18" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="1">
+        <v>100</v>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="J18" s="6"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="U18" s="1"/>
+      <c r="V18" s="1"/>
+      <c r="W18" s="11"/>
+      <c r="X18" s="1"/>
+      <c r="Y18" s="1"/>
+      <c r="Z18" s="1"/>
+    </row>
+    <row r="19" ht="42.75">
+      <c r="A19" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="1">
+        <v>100</v>
+      </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="J19" s="1"/>
+      <c r="K19" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="L19" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="M19" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="N19" s="18"/>
+      <c r="O19" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="V19" s="1"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="1"/>
+      <c r="Y19" s="1"/>
+      <c r="Z19" s="1"/>
+    </row>
+    <row r="20" ht="33.75">
+      <c r="A20" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="1">
+        <v>100</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="H20" s="11"/>
+      <c r="I20" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="J20" t="s">
+        <v>125</v>
+      </c>
+      <c r="K20" s="6"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="11"/>
+      <c r="V20" s="1"/>
+      <c r="W20" s="11"/>
+      <c r="X20" s="1"/>
+      <c r="Y20" s="1"/>
+      <c r="Z20" s="1"/>
+    </row>
+    <row r="21" ht="33.75">
+      <c r="A21" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="1">
+        <v>100</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="H21" s="11"/>
+      <c r="I21" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="J21" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="K21" s="6"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="18"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="11"/>
+      <c r="V21" s="1"/>
+      <c r="W21" s="11"/>
+      <c r="X21" s="1"/>
+      <c r="Y21" s="1"/>
+      <c r="Z21" s="1"/>
+    </row>
+    <row r="22" ht="22.5">
+      <c r="A22" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="1">
+        <v>100</v>
+      </c>
+      <c r="G22" s="12"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J22" s="1"/>
+      <c r="K22" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="L22" s="17"/>
+      <c r="M22" s="18"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1"/>
+      <c r="U22" s="11"/>
+      <c r="V22" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="W22" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="X22" s="1"/>
+      <c r="Y22" s="1"/>
+      <c r="Z22" s="1"/>
+    </row>
+    <row r="23" ht="28.5">
+      <c r="A23" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="1">
+        <v>100</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="H23" s="11"/>
+      <c r="I23" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J23" s="1"/>
+      <c r="K23" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="M23" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="N23" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="O23" s="12"/>
+      <c r="P23" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="1">
+        <v>546455</v>
+      </c>
+      <c r="T23" s="1"/>
+      <c r="U23" s="11"/>
+      <c r="V23" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="W23" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="X23" s="1"/>
+      <c r="Y23" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z23" s="21" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="1">
+        <v>100</v>
+      </c>
+      <c r="G24" s="11"/>
+      <c r="H24" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="11"/>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="11"/>
+      <c r="S24" s="11"/>
+      <c r="T24" s="11"/>
+      <c r="U24" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="V24" s="11"/>
+      <c r="W24" s="11"/>
+      <c r="X24" s="11"/>
+      <c r="Y24" s="11"/>
+      <c r="Z24" s="11"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" t="s">
+        <v>150</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="1">
+        <v>100</v>
+      </c>
+      <c r="G25" s="11"/>
+      <c r="H25" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="11"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="11"/>
+      <c r="R25" s="11"/>
+      <c r="S25" s="11"/>
+      <c r="T25" s="11"/>
+      <c r="U25" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="V25" s="11"/>
+      <c r="W25" s="11"/>
+      <c r="X25" s="11"/>
+      <c r="Y25" s="11"/>
+      <c r="Z25" s="11"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="Z23"/>
+  </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
@@ -1148,31 +2900,160 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="17.7109375"/>
-    <col customWidth="1" min="3" max="3" width="29.140625"/>
+    <col customWidth="1" min="1" max="1" width="14.140625"/>
+    <col customWidth="1" min="2" max="2" width="27.7109375"/>
+    <col customWidth="1" min="3" max="3" width="13.7109375"/>
+    <col customWidth="1" min="4" max="4" width="18.421875"/>
+    <col customWidth="1" min="5" max="5" width="15.00390625"/>
+    <col customWidth="1" min="7" max="7" width="22.7109375"/>
+    <col customWidth="1" min="8" max="9" width="20.8515625"/>
+    <col customWidth="1" min="10" max="10" width="21.00390625"/>
+    <col customWidth="1" min="11" max="14" width="22.8515625"/>
+    <col customWidth="1" min="15" max="15" width="25.7109375"/>
+    <col bestFit="1" min="17" max="17" width="11.28125"/>
+    <col customWidth="1" min="18" max="18" width="19.8515625"/>
+    <col customWidth="1" min="23" max="23" width="21.8515625"/>
+    <col customWidth="1" min="24" max="24" width="14.28125"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
         <v>15</v>
       </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>26</v>
+      </c>
+      <c r="R1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" t="s">
+        <v>28</v>
+      </c>
+      <c r="T1" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA1"/>
+    </row>
+    <row r="2" ht="28.5">
+      <c r="A2" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="1">
+        <v>100</v>
+      </c>
+      <c r="G2" s="13"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="M2" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -1186,37 +3067,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.421875"/>
-    <col customWidth="1" min="3" max="3" width="21.421875"/>
-    <col customWidth="1" min="4" max="4" width="27.28125"/>
+    <col customWidth="1" min="1" max="1" width="20.00390625"/>
+    <col customWidth="1" min="2" max="2" width="43.421875"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1231,35 +3099,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="25.8515625"/>
+    <col customWidth="1" min="1" max="1" width="20.7109375"/>
+    <col customWidth="1" min="2" max="2" width="53.00390625"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>158</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -1274,31 +3131,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="29.421875"/>
-    <col customWidth="1" min="2" max="2" width="26.140625"/>
-    <col customWidth="1" min="3" max="3" width="20.57421875"/>
+    <col customWidth="1" min="1" max="1" width="38.7109375"/>
+    <col customWidth="1" min="2" max="2" width="52.00390625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" t="s">
-        <v>25</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>28</v>
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified Billers data provider and test data
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="23"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -24,13 +24,19 @@
     <sheet name="DashboardLoanValidation" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="DashboardRVTPaymentPopup" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="DashboardAccountPortfolio" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="SettingsPanelUserData" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="LoginDataSettings" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="PasswordChangeDataSettings" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="AccountSuccessMessageSettings" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="LoginAfteThePasswordChange" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="SuccessMessageSettings" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="212">
   <si>
     <t>userName</t>
   </si>
@@ -639,6 +645,33 @@
   </si>
   <si>
     <t>200</t>
+  </si>
+  <si>
+    <t>settingsUserDetails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safras|95-c , Old Post Office Road , Sainthamaruthu -10|N/A|Kalmunai|Sri Lanka|853231592V</t>
+  </si>
+  <si>
+    <t>safras77</t>
+  </si>
+  <si>
+    <t>newPassword</t>
+  </si>
+  <si>
+    <t>Hoax@2345</t>
+  </si>
+  <si>
+    <t>primaryAccountSentSuccessMsg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary Account Set Successful</t>
+  </si>
+  <si>
+    <t>LoginErrorMessage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS: 4</t>
   </si>
 </sst>
 </file>
@@ -689,23 +722,12 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="16">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -713,13 +735,9 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -735,13 +753,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -750,6 +762,9 @@
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1282,7 +1297,7 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1441,13 +1456,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="4" t="s">
         <v>174</v>
       </c>
     </row>
@@ -1470,19 +1485,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="12" t="s">
         <v>178</v>
       </c>
     </row>
@@ -1493,13 +1508,13 @@
       <c r="B2" t="s">
         <v>180</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="4" t="s">
         <v>183</v>
       </c>
     </row>
@@ -1521,24 +1536,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="12" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" ht="67.5" customHeight="1">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="13" t="s">
         <v>188</v>
       </c>
     </row>
@@ -1561,36 +1576,36 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="12" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="4" t="s">
         <v>196</v>
       </c>
     </row>
@@ -1651,8 +1666,33 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="4" t="s">
         <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="32.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="2" ht="57">
+      <c r="A2" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -1690,8 +1730,164 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="20.28125"/>
+    <col customWidth="1" min="2" max="2" width="17.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="29.421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="39.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="15.140625"/>
   </cols>
@@ -1759,13 +1955,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1825,13 +2021,13 @@
       <c r="K1" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="2" t="s">
         <v>23</v>
       </c>
       <c r="O1" t="s">
@@ -1846,7 +2042,7 @@
       <c r="R1" t="s">
         <v>27</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="2" t="s">
         <v>28</v>
       </c>
       <c r="T1" t="s">
@@ -1858,7 +2054,7 @@
       <c r="V1" t="s">
         <v>31</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="2" t="s">
         <v>32</v>
       </c>
       <c r="X1" s="1" t="s">
@@ -1875,7 +2071,7 @@
       <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C2" t="s">
@@ -1890,21 +2086,21 @@
       <c r="F2">
         <v>100</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C3" t="s">
@@ -1919,7 +2115,7 @@
       <c r="F3">
         <v>100</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="4" t="s">
         <v>44</v>
       </c>
       <c r="I3" t="s">
@@ -1930,10 +2126,10 @@
       </c>
     </row>
     <row r="4" ht="28.5">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C4" t="s">
@@ -1948,7 +2144,7 @@
       <c r="F4">
         <v>100</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="4" t="s">
         <v>47</v>
       </c>
       <c r="I4" t="s">
@@ -1959,10 +2155,10 @@
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>49</v>
       </c>
       <c r="C5" t="s">
@@ -1977,7 +2173,7 @@
       <c r="F5">
         <v>100</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="4" t="s">
         <v>47</v>
       </c>
       <c r="I5" t="s">
@@ -1991,7 +2187,7 @@
       <c r="A6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -2006,24 +2202,24 @@
       <c r="F6" s="1">
         <v>100</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
@@ -2044,7 +2240,7 @@
       <c r="F7" s="1">
         <v>100</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="4" t="s">
         <v>58</v>
       </c>
       <c r="I7" t="s">
@@ -2055,10 +2251,10 @@
       </c>
     </row>
     <row r="8" ht="28.5">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -2073,32 +2269,32 @@
       <c r="F8" s="1">
         <v>100</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="6" t="s">
+      <c r="G8" s="4"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
       <c r="P8" t="s">
         <v>64</v>
       </c>
-      <c r="Q8" s="13" t="s">
+      <c r="Q8" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" ht="28.5">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -2113,27 +2309,27 @@
       <c r="F9" s="1">
         <v>100</v>
       </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="6" t="s">
+      <c r="G9" s="4"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="11" t="s">
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="4" t="s">
         <v>69</v>
       </c>
       <c r="P9" t="s">
         <v>64</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="Q9" s="4" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2141,7 +2337,7 @@
       <c r="A10" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="3" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -2156,30 +2352,30 @@
       <c r="F10" s="1">
         <v>100</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="6" t="s">
+      <c r="G10" s="4"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="M10" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N10" s="6"/>
-      <c r="O10" s="11"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="4"/>
       <c r="P10" t="s">
         <v>64</v>
       </c>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11" t="s">
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4" t="s">
         <v>77</v>
       </c>
       <c r="S10" t="s">
@@ -2193,7 +2389,7 @@
       <c r="A11" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -2208,26 +2404,26 @@
       <c r="F11" s="1">
         <v>100</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="16" t="s">
+      <c r="G11" s="4"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6" t="s">
+      <c r="J11" s="3"/>
+      <c r="K11" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="11"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="4"/>
       <c r="P11" t="s">
         <v>64</v>
       </c>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11" t="s">
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4" t="s">
         <v>81</v>
       </c>
       <c r="S11" t="s">
@@ -2241,7 +2437,7 @@
       <c r="A12" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>83</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -2256,32 +2452,29 @@
       <c r="F12" s="1">
         <v>100</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H12" s="12"/>
-      <c r="I12" s="16" t="s">
+      <c r="H12" s="5"/>
+      <c r="I12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="11"/>
-      <c r="P12"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-      <c r="S12"/>
-      <c r="T12"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
     </row>
     <row r="13" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="3" t="s">
         <v>86</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -2296,19 +2489,19 @@
       <c r="F13" s="1">
         <v>100</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="4" t="s">
         <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>53</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="I13" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2316,7 +2509,7 @@
       <c r="A14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -2331,22 +2524,22 @@
       <c r="F14" s="1">
         <v>100</v>
       </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="13" t="s">
+      <c r="G14" s="4"/>
+      <c r="H14" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1" t="s">
         <v>94</v>
@@ -2360,7 +2553,7 @@
       <c r="A15" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B15" s="6"/>
+      <c r="B15" s="3"/>
       <c r="C15" s="1" t="s">
         <v>38</v>
       </c>
@@ -2373,20 +2566,20 @@
       <c r="F15" s="1">
         <v>100</v>
       </c>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11" t="s">
+      <c r="G15" s="4"/>
+      <c r="H15" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="I15" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1" t="s">
         <v>94</v>
@@ -2403,7 +2596,7 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="10" t="s">
         <v>98</v>
       </c>
       <c r="B16" t="s">
@@ -2421,7 +2614,7 @@
       <c r="F16" s="1">
         <v>100</v>
       </c>
-      <c r="H16" s="13" t="s">
+      <c r="H16" s="4" t="s">
         <v>100</v>
       </c>
       <c r="I16" t="s">
@@ -2431,11 +2624,11 @@
         <v>101</v>
       </c>
     </row>
-    <row r="17" s="11" customFormat="1" ht="42.75">
-      <c r="A17" s="19" t="s">
+    <row r="17" s="4" customFormat="1" ht="42.75">
+      <c r="A17" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>103</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -2450,23 +2643,23 @@
       <c r="F17" s="1">
         <v>100</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="11"/>
-      <c r="I17" s="6" t="s">
+      <c r="H17" s="4"/>
+      <c r="I17" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="J17" s="6"/>
-      <c r="K17" s="18" t="s">
+      <c r="J17" s="3"/>
+      <c r="K17" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="L17" s="18" t="s">
+      <c r="L17" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="12" t="s">
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="5" t="s">
         <v>108</v>
       </c>
       <c r="P17" s="1"/>
@@ -2476,7 +2669,7 @@
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
-      <c r="W17" s="11" t="s">
+      <c r="W17" s="4" t="s">
         <v>109</v>
       </c>
       <c r="X17" s="1"/>
@@ -2484,10 +2677,10 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" ht="56.25">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="3" t="s">
         <v>111</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -2502,17 +2695,17 @@
       <c r="F18" s="1">
         <v>100</v>
       </c>
-      <c r="G18" s="12"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="16" t="s">
+      <c r="G18" s="5"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="J18" s="6"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="12" t="s">
+      <c r="J18" s="3"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="5" t="s">
         <v>108</v>
       </c>
       <c r="P18" s="1"/>
@@ -2524,16 +2717,16 @@
       </c>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
-      <c r="W18" s="11"/>
+      <c r="W18" s="4"/>
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
     </row>
     <row r="19" ht="42.75">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="3" t="s">
         <v>114</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -2548,48 +2741,48 @@
       <c r="F19" s="1">
         <v>100</v>
       </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="16" t="s">
+      <c r="G19" s="5"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="7" t="s">
         <v>115</v>
       </c>
       <c r="J19" s="1"/>
-      <c r="K19" s="6" t="s">
+      <c r="K19" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="L19" s="17" t="s">
+      <c r="L19" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="M19" s="18" t="s">
+      <c r="M19" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="N19" s="18"/>
-      <c r="O19" s="12" t="s">
+      <c r="N19" s="9"/>
+      <c r="O19" s="5" t="s">
         <v>108</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>119</v>
       </c>
       <c r="Q19" s="1"/>
-      <c r="R19" s="20" t="s">
+      <c r="R19" s="5" t="s">
         <v>120</v>
       </c>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
-      <c r="U19" s="11" t="s">
+      <c r="U19" s="4" t="s">
         <v>121</v>
       </c>
       <c r="V19" s="1"/>
-      <c r="W19" s="11"/>
+      <c r="W19" s="4"/>
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
     </row>
     <row r="20" ht="33.75">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="3" t="s">
         <v>123</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -2604,38 +2797,38 @@
       <c r="F20" s="1">
         <v>100</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="16" t="s">
+      <c r="H20" s="4"/>
+      <c r="I20" s="7" t="s">
         <v>125</v>
       </c>
       <c r="J20" t="s">
         <v>125</v>
       </c>
-      <c r="K20" s="6"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="12"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="5"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
-      <c r="R20" s="12"/>
+      <c r="R20" s="5"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
-      <c r="U20" s="11"/>
+      <c r="U20" s="4"/>
       <c r="V20" s="1"/>
-      <c r="W20" s="11"/>
+      <c r="W20" s="4"/>
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
     </row>
     <row r="21" ht="33.75">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="3" t="s">
         <v>126</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -2650,38 +2843,38 @@
       <c r="F21" s="1">
         <v>100</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="16" t="s">
+      <c r="H21" s="4"/>
+      <c r="I21" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="K21" s="6"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="12"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="5"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
-      <c r="R21" s="12"/>
+      <c r="R21" s="5"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
-      <c r="U21" s="11"/>
+      <c r="U21" s="4"/>
       <c r="V21" s="1"/>
-      <c r="W21" s="11"/>
+      <c r="W21" s="4"/>
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
     </row>
     <row r="22" ht="22.5">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="3" t="s">
         <v>130</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -2696,29 +2889,29 @@
       <c r="F22" s="1">
         <v>100</v>
       </c>
-      <c r="G22" s="12"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="16" t="s">
+      <c r="G22" s="5"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="7" t="s">
         <v>131</v>
       </c>
       <c r="J22" s="1"/>
-      <c r="K22" s="19" t="s">
+      <c r="K22" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="L22" s="17"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="12"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="5"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
-      <c r="R22" s="12"/>
+      <c r="R22" s="5"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="11" t="s">
+      <c r="U22" s="4"/>
+      <c r="V22" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="W22" s="11" t="s">
+      <c r="W22" s="4" t="s">
         <v>134</v>
       </c>
       <c r="X22" s="1"/>
@@ -2726,10 +2919,10 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" ht="28.5">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="3" t="s">
         <v>136</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -2744,48 +2937,48 @@
       <c r="F23" s="1">
         <v>100</v>
       </c>
-      <c r="G23" s="12" t="s">
+      <c r="G23" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="16" t="s">
+      <c r="H23" s="4"/>
+      <c r="I23" s="7" t="s">
         <v>138</v>
       </c>
       <c r="J23" s="1"/>
-      <c r="K23" s="19" t="s">
+      <c r="K23" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="L23" s="17" t="s">
+      <c r="L23" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="M23" s="18" t="s">
+      <c r="M23" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="N23" s="18" t="s">
+      <c r="N23" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="O23" s="12"/>
+      <c r="O23" s="5"/>
       <c r="P23" s="1" t="s">
         <v>143</v>
       </c>
       <c r="Q23" s="1"/>
-      <c r="R23" s="12"/>
+      <c r="R23" s="5"/>
       <c r="S23" s="1">
         <v>546455</v>
       </c>
       <c r="T23" s="1"/>
-      <c r="U23" s="11"/>
-      <c r="V23" s="11" t="s">
+      <c r="U23" s="4"/>
+      <c r="V23" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="W23" s="11" t="s">
+      <c r="W23" s="4" t="s">
         <v>134</v>
       </c>
       <c r="X23" s="1"/>
       <c r="Y23" t="s">
         <v>144</v>
       </c>
-      <c r="Z23" s="21" t="s">
+      <c r="Z23" s="11" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2793,7 +2986,7 @@
       <c r="A24" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="4"/>
       <c r="C24" s="1" t="s">
         <v>38</v>
       </c>
@@ -2806,42 +2999,42 @@
       <c r="F24" s="1">
         <v>100</v>
       </c>
-      <c r="G24" s="11"/>
-      <c r="H24" s="13" t="s">
+      <c r="G24" s="4"/>
+      <c r="H24" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="J24" s="13" t="s">
+      <c r="J24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K24" s="13" t="s">
+      <c r="K24" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
-      <c r="R24" s="11"/>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-      <c r="U24" s="13" t="s">
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="V24" s="11"/>
-      <c r="W24" s="11"/>
-      <c r="X24" s="11"/>
-      <c r="Y24" s="11"/>
-      <c r="Z24" s="11"/>
+      <c r="V24" s="4"/>
+      <c r="W24" s="4"/>
+      <c r="X24" s="4"/>
+      <c r="Y24" s="4"/>
+      <c r="Z24" s="4"/>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" t="s">
         <v>150</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="4"/>
       <c r="C25" s="1" t="s">
         <v>38</v>
       </c>
@@ -2854,36 +3047,36 @@
       <c r="F25" s="1">
         <v>100</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="13" t="s">
+      <c r="G25" s="4"/>
+      <c r="H25" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="I25" s="13" t="s">
+      <c r="I25" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="J25" s="13" t="s">
+      <c r="J25" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="K25" s="13" t="s">
+      <c r="K25" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="13" t="s">
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="V25" s="11"/>
-      <c r="W25" s="11"/>
-      <c r="X25" s="11"/>
-      <c r="Y25" s="11"/>
-      <c r="Z25" s="11"/>
+      <c r="V25" s="4"/>
+      <c r="W25" s="4"/>
+      <c r="X25" s="4"/>
+      <c r="Y25" s="4"/>
+      <c r="Z25" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2944,19 +3137,19 @@
       <c r="I1" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="2" t="s">
         <v>23</v>
       </c>
       <c r="O1" t="s">
@@ -2995,16 +3188,15 @@
       <c r="Z1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AA1"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -3016,30 +3208,30 @@
       <c r="F2" s="1">
         <v>100</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="6" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N2" s="15"/>
-      <c r="O2" s="11"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="4"/>
       <c r="P2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13" t="s">
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4" t="s">
         <v>77</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -3048,9 +3240,9 @@
       <c r="T2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>

</xml_diff>

<commit_message>
Changes to transfers and billers
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="28"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -29,14 +29,21 @@
     <sheet name="PasswordChangeDataSettings" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="AccountSuccessMessageSettings" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="LoginAfteThePasswordChange" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="SuccessMessageSettings" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="AccountPreviewDetailsSavingsFD" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="SuccessMessageSettings" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="AmountSavingsFD" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="LoginDataSavingsFD" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="AccountNumberSavingsFD" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="OwnAccountTransferData" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="OtherAccountTransfersData" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="OtherCreditCardTransferData" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
   <si>
     <t>userName</t>
   </si>
@@ -650,10 +657,10 @@
     <t>settingsUserDetails</t>
   </si>
   <si>
-    <t xml:space="preserve">Safras|95-c , Old Post Office Road , Sainthamaruthu -10|N/A|Kalmunai|Sri Lanka|853231592V</t>
-  </si>
-  <si>
-    <t>safras77</t>
+    <t xml:space="preserve">Mohan|517/10 Mattegoda|N/A|Mattegoda|Sri Lanka|910881647V</t>
+  </si>
+  <si>
+    <t>mohanw</t>
   </si>
   <si>
     <t>newPassword</t>
@@ -672,13 +679,188 @@
   </si>
   <si>
     <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS: 4</t>
+  </si>
+  <si>
+    <t>DetailsSavingsFD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sampath Sanhinda Saver|TestUser100|016751000165|BUSINESS TRANSACTIONS|SALES AND BUSINESS TURNOVER</t>
+  </si>
+  <si>
+    <t>nickName</t>
+  </si>
+  <si>
+    <t>TestUser100</t>
+  </si>
+  <si>
+    <t>shirania</t>
+  </si>
+  <si>
+    <t>016751000165</t>
+  </si>
+  <si>
+    <t>errorMsg1</t>
+  </si>
+  <si>
+    <t>errorMsg2</t>
+  </si>
+  <si>
+    <t>minAmount</t>
+  </si>
+  <si>
+    <t>maxAmount</t>
+  </si>
+  <si>
+    <t>minAmountMsg</t>
+  </si>
+  <si>
+    <t>maxAmountMsg</t>
+  </si>
+  <si>
+    <t>noAmount</t>
+  </si>
+  <si>
+    <t>errMinimumTransferAmount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To Account is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowed Minimum transaction amount is 15.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowed Maximum transaction amount is 50000.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0167 5100 0152</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum transfer amount must be greater than Rs.0</t>
+  </si>
+  <si>
+    <t>errorMsgInsufficientFunds</t>
+  </si>
+  <si>
+    <t>minAmountEntry</t>
+  </si>
+  <si>
+    <t>maxAmountEntry</t>
+  </si>
+  <si>
+    <t>receiverName</t>
+  </si>
+  <si>
+    <t>bankName</t>
+  </si>
+  <si>
+    <t>actualTransactionAmount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">actualTransactionAmount
+Insufficient funds in the selected account</t>
+  </si>
+  <si>
+    <t>2550040541</t>
+  </si>
+  <si>
+    <t>Baabu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit Income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMPATH BANK PLC - COMPANY NO PQ 144</t>
+  </si>
+  <si>
+    <t>errCreditCardNumberRequired</t>
+  </si>
+  <si>
+    <t>errReEnterCreditCardNumberRequired</t>
+  </si>
+  <si>
+    <t>errNameOnCardRequired</t>
+  </si>
+  <si>
+    <t>errBankRequired</t>
+  </si>
+  <si>
+    <t>errAmountRequired</t>
+  </si>
+  <si>
+    <t>errPurposeRequired</t>
+  </si>
+  <si>
+    <t>errBeneficiaryRemarkRequired</t>
+  </si>
+  <si>
+    <t>creditCardNumber</t>
+  </si>
+  <si>
+    <t>reEnterCardNumber</t>
+  </si>
+  <si>
+    <t>nameOnCard</t>
+  </si>
+  <si>
+    <t>branchName</t>
+  </si>
+  <si>
+    <t>mdtAmount</t>
+  </si>
+  <si>
+    <t>errorMessageMaxTransactionLimit</t>
+  </si>
+  <si>
+    <t>errInsufficientfunds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credit Card Number/CAN is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-enter Credit Card Number/CAN is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name On Card is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select Purpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beneficiary Remark is required</t>
+  </si>
+  <si>
+    <t>376657973920377</t>
+  </si>
+  <si>
+    <t>Supun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NATIONS TRUST BANK</t>
+  </si>
+  <si>
+    <t>BADULLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowed Maximum transaction amount is 30000.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -699,6 +881,20 @@
     <font>
       <sz val="10.000000"/>
       <color rgb="FF6AAB73"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
+      <color rgb="FF067D17"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -722,11 +918,8 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -738,9 +931,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
       <protection hidden="0" locked="1"/>
@@ -769,8 +959,30 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1303,7 +1515,7 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1324,21 +1536,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
@@ -1406,10 +1618,10 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1420,10 +1632,10 @@
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
@@ -1462,13 +1674,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>174</v>
       </c>
     </row>
@@ -1491,19 +1703,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="12" t="s">
         <v>178</v>
       </c>
     </row>
@@ -1514,13 +1726,13 @@
       <c r="B2" t="s">
         <v>180</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>183</v>
       </c>
     </row>
@@ -1542,24 +1754,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" ht="67.5" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>188</v>
       </c>
     </row>
@@ -1582,36 +1794,36 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="12" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>196</v>
       </c>
     </row>
@@ -1672,7 +1884,7 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>202</v>
       </c>
     </row>
@@ -1692,12 +1904,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="2" ht="57">
-      <c r="A2" s="5" t="s">
+    <row r="2" ht="42.75">
+      <c r="A2" s="4" t="s">
         <v>204</v>
       </c>
     </row>
@@ -1719,24 +1931,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1753,24 +1965,24 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1791,18 +2003,18 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>207</v>
       </c>
     </row>
@@ -1822,12 +2034,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>209</v>
       </c>
     </row>
@@ -1842,32 +2054,41 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="15.57421875"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1882,18 +2103,226 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" s="5" customFormat="1">
+      <c r="A2" s="5" t="s">
+        <v>213</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="39.57421875"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="2" t="s">
         <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1000</v>
+      </c>
+      <c r="B2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="14.140625"/>
+    <col customWidth="1" min="2" max="2" width="13.8515625"/>
+    <col customWidth="1" min="3" max="3" width="14.421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="28.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="27.7109375"/>
+    <col customWidth="1" min="2" max="2" width="18.57421875"/>
+    <col customWidth="1" min="3" max="3" width="13.421875"/>
+    <col customWidth="1" min="4" max="4" width="12.140625"/>
+    <col customWidth="1" min="5" max="5" width="44.57421875"/>
+    <col customWidth="1" min="6" max="6" width="17.00390625"/>
+    <col customWidth="1" min="7" max="7" width="12.140625"/>
+    <col customWidth="1" min="9" max="9" width="15.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="57">
+      <c r="A1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" ht="85.5">
+      <c r="A2" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C2" s="5">
+        <v>14</v>
+      </c>
+      <c r="D2" s="5">
+        <v>50001</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="17">
+        <v>0</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1913,25 +2342,260 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="23.421875"/>
+    <col customWidth="1" min="2" max="2" width="11.421875"/>
+    <col customWidth="1" min="5" max="5" width="24.8515625"/>
+    <col customWidth="1" min="6" max="6" width="20.421875"/>
+    <col bestFit="1" min="7" max="7" width="10.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>236</v>
+      </c>
+      <c r="J1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" ht="42.75">
+      <c r="A2" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>50001</v>
+      </c>
+      <c r="D2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="L2" s="5">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="8" max="8" width="24.7109375"/>
+    <col customWidth="1" min="9" max="9" width="33.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="4" customFormat="1" ht="57">
+      <c r="A1" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" s="4" customFormat="1" ht="114">
+      <c r="A2" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>227</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>264</v>
+      </c>
+      <c r="J2" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="K2" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="L2" s="22" t="s">
+        <v>267</v>
+      </c>
+      <c r="M2" s="22">
+        <v>30001</v>
+      </c>
+      <c r="N2" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="O2" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q2" s="22">
+        <v>501</v>
+      </c>
+      <c r="R2" s="22">
+        <v>0</v>
+      </c>
+      <c r="S2" s="23" t="s">
+        <v>269</v>
+      </c>
+      <c r="T2" s="23" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1950,24 +2614,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2027,13 +2691,13 @@
       <c r="K1" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>23</v>
       </c>
       <c r="O1" t="s">
@@ -2048,28 +2712,28 @@
       <c r="R1" t="s">
         <v>27</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="3" t="s">
         <v>28</v>
       </c>
       <c r="T1" t="s">
         <v>29</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>30</v>
       </c>
       <c r="V1" t="s">
         <v>31</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="W1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="2" t="s">
         <v>33</v>
       </c>
       <c r="Y1" t="s">
         <v>34</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2077,7 +2741,7 @@
       <c r="A2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C2" t="s">
@@ -2092,21 +2756,21 @@
       <c r="F2">
         <v>100</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C3" t="s">
@@ -2121,7 +2785,7 @@
       <c r="F3">
         <v>100</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>44</v>
       </c>
       <c r="I3" t="s">
@@ -2132,10 +2796,10 @@
       </c>
     </row>
     <row r="4" ht="28.5">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>46</v>
       </c>
       <c r="C4" t="s">
@@ -2150,7 +2814,7 @@
       <c r="F4">
         <v>100</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>47</v>
       </c>
       <c r="I4" t="s">
@@ -2161,10 +2825,10 @@
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C5" t="s">
@@ -2179,7 +2843,7 @@
       <c r="F5">
         <v>100</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>47</v>
       </c>
       <c r="I5" t="s">
@@ -2190,42 +2854,42 @@
       </c>
     </row>
     <row r="6" ht="42.75">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>100</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
@@ -2234,19 +2898,19 @@
       <c r="B7" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <v>100</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="5" t="s">
         <v>58</v>
       </c>
       <c r="I7" t="s">
@@ -2257,85 +2921,85 @@
       </c>
     </row>
     <row r="8" ht="28.5">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>100</v>
       </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="5" t="s">
+      <c r="G8" s="5"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
       <c r="P8" t="s">
         <v>64</v>
       </c>
-      <c r="Q8" s="6" t="s">
+      <c r="Q8" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" ht="28.5">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>100</v>
       </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="5" t="s">
+      <c r="G9" s="5"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="6" t="s">
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="5" t="s">
         <v>69</v>
       </c>
       <c r="P9" t="s">
         <v>64</v>
       </c>
-      <c r="Q9" s="6" t="s">
+      <c r="Q9" s="5" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2343,45 +3007,45 @@
       <c r="A10" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>100</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="5" t="s">
+      <c r="G10" s="5"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="K10" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L10" s="5" t="s">
+      <c r="L10" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="M10" s="5" t="s">
+      <c r="M10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="N10" s="5"/>
-      <c r="O10" s="6"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="5"/>
       <c r="P10" t="s">
         <v>64</v>
       </c>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6" t="s">
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5" t="s">
         <v>77</v>
       </c>
       <c r="S10" t="s">
@@ -2395,41 +3059,41 @@
       <c r="A11" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <v>100</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="9" t="s">
+      <c r="G11" s="5"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5" t="s">
+      <c r="J11" s="4"/>
+      <c r="K11" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="L11" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="6"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="5"/>
       <c r="P11" t="s">
         <v>64</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6" t="s">
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5" t="s">
         <v>81</v>
       </c>
       <c r="S11" t="s">
@@ -2443,184 +3107,184 @@
       <c r="A12" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
         <v>100</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="9" t="s">
+      <c r="H12" s="1"/>
+      <c r="I12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
     </row>
     <row r="13" ht="42.75">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="2">
         <v>100</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="5" t="s">
         <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>53</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="J13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="4" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="14" ht="45">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="2">
         <v>100</v>
       </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6" t="s">
+      <c r="G14" s="5"/>
+      <c r="H14" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="J14" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="K14" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3" t="s">
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
     </row>
     <row r="15" ht="33.75">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="3" t="s">
+      <c r="B15" s="4"/>
+      <c r="C15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <v>100</v>
       </c>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6" t="s">
+      <c r="G15" s="5"/>
+      <c r="H15" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="J15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="9"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3" t="s">
+      <c r="K15" s="7"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-      <c r="Y15" s="3"/>
-      <c r="Z15" s="3"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="2"/>
+      <c r="Z15" s="2"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="10" t="s">
         <v>98</v>
       </c>
       <c r="B16" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="2">
         <v>100</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="5" t="s">
         <v>100</v>
       </c>
       <c r="I16" t="s">
@@ -2630,361 +3294,361 @@
         <v>101</v>
       </c>
     </row>
-    <row r="17" s="6" customFormat="1" ht="42.75">
-      <c r="A17" s="12" t="s">
+    <row r="17" s="5" customFormat="1" ht="42.75">
+      <c r="A17" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="2">
         <v>100</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="6"/>
-      <c r="I17" s="5" t="s">
+      <c r="H17" s="5"/>
+      <c r="I17" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="11" t="s">
+      <c r="J17" s="4"/>
+      <c r="K17" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="L17" s="11" t="s">
+      <c r="L17" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="7" t="s">
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="6" t="s">
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="2"/>
+      <c r="W17" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="X17" s="3"/>
-      <c r="Y17" s="3"/>
-      <c r="Z17" s="3"/>
+      <c r="X17" s="2"/>
+      <c r="Y17" s="2"/>
+      <c r="Z17" s="2"/>
     </row>
     <row r="18" ht="56.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="2">
         <v>100</v>
       </c>
-      <c r="G18" s="7"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="9" t="s">
+      <c r="G18" s="1"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="7" t="s">
+      <c r="J18" s="4"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3" t="s">
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="6"/>
-      <c r="X18" s="3"/>
-      <c r="Y18" s="3"/>
-      <c r="Z18" s="3"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="5"/>
+      <c r="X18" s="2"/>
+      <c r="Y18" s="2"/>
+      <c r="Z18" s="2"/>
     </row>
     <row r="19" ht="42.75">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="2">
         <v>100</v>
       </c>
-      <c r="G19" s="7"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="9" t="s">
+      <c r="G19" s="1"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="J19" s="3"/>
-      <c r="K19" s="5" t="s">
+      <c r="J19" s="2"/>
+      <c r="K19" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="M19" s="11" t="s">
+      <c r="M19" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="N19" s="11"/>
-      <c r="O19" s="7" t="s">
+      <c r="N19" s="9"/>
+      <c r="O19" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="P19" s="3" t="s">
+      <c r="P19" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="7" t="s">
+      <c r="Q19" s="2"/>
+      <c r="R19" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="6" t="s">
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="V19" s="3"/>
-      <c r="W19" s="6"/>
-      <c r="X19" s="3"/>
-      <c r="Y19" s="3"/>
-      <c r="Z19" s="3"/>
+      <c r="V19" s="2"/>
+      <c r="W19" s="5"/>
+      <c r="X19" s="2"/>
+      <c r="Y19" s="2"/>
+      <c r="Z19" s="2"/>
     </row>
     <row r="20" ht="33.75">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="2">
         <v>100</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="6"/>
-      <c r="I20" s="9" t="s">
+      <c r="H20" s="5"/>
+      <c r="I20" s="7" t="s">
         <v>125</v>
       </c>
       <c r="J20" t="s">
         <v>125</v>
       </c>
-      <c r="K20" s="5"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="6"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="6"/>
-      <c r="X20" s="3"/>
-      <c r="Y20" s="3"/>
-      <c r="Z20" s="3"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="5"/>
+      <c r="V20" s="2"/>
+      <c r="W20" s="5"/>
+      <c r="X20" s="2"/>
+      <c r="Y20" s="2"/>
+      <c r="Z20" s="2"/>
     </row>
     <row r="21" ht="33.75">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="2">
         <v>100</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="6"/>
-      <c r="I21" s="9" t="s">
+      <c r="H21" s="5"/>
+      <c r="I21" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="J21" s="12" t="s">
+      <c r="J21" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="K21" s="5"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="6"/>
-      <c r="X21" s="3"/>
-      <c r="Y21" s="3"/>
-      <c r="Z21" s="3"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="5"/>
+      <c r="V21" s="2"/>
+      <c r="W21" s="5"/>
+      <c r="X21" s="2"/>
+      <c r="Y21" s="2"/>
+      <c r="Z21" s="2"/>
     </row>
     <row r="22" ht="22.5">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="2">
         <v>100</v>
       </c>
-      <c r="G22" s="7"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="9" t="s">
+      <c r="G22" s="1"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="J22" s="3"/>
-      <c r="K22" s="12" t="s">
+      <c r="J22" s="2"/>
+      <c r="K22" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="L22" s="10"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="7"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-      <c r="U22" s="6"/>
-      <c r="V22" s="6" t="s">
+      <c r="L22" s="8"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="W22" s="6" t="s">
+      <c r="W22" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="X22" s="3"/>
-      <c r="Y22" s="3"/>
-      <c r="Z22" s="3"/>
+      <c r="X22" s="2"/>
+      <c r="Y22" s="2"/>
+      <c r="Z22" s="2"/>
     </row>
     <row r="23" ht="28.5">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="2">
         <v>100</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="H23" s="6"/>
-      <c r="I23" s="9" t="s">
+      <c r="H23" s="5"/>
+      <c r="I23" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="J23" s="3"/>
-      <c r="K23" s="12" t="s">
+      <c r="J23" s="2"/>
+      <c r="K23" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="L23" s="10" t="s">
+      <c r="L23" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="M23" s="11" t="s">
+      <c r="M23" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="N23" s="11" t="s">
+      <c r="N23" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="O23" s="7"/>
-      <c r="P23" s="3" t="s">
+      <c r="O23" s="1"/>
+      <c r="P23" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="7"/>
-      <c r="S23" s="3">
+      <c r="Q23" s="2"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="2">
         <v>546455</v>
       </c>
-      <c r="T23" s="3"/>
-      <c r="U23" s="6"/>
-      <c r="V23" s="6" t="s">
+      <c r="T23" s="2"/>
+      <c r="U23" s="5"/>
+      <c r="V23" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="W23" s="6" t="s">
+      <c r="W23" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="X23" s="3"/>
+      <c r="X23" s="2"/>
       <c r="Y23" t="s">
         <v>144</v>
       </c>
-      <c r="Z23" s="13" t="s">
+      <c r="Z23" s="11" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2992,97 +3656,97 @@
       <c r="A24" t="s">
         <v>146</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="3" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="2">
         <v>100</v>
       </c>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6" t="s">
+      <c r="G24" s="5"/>
+      <c r="H24" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="J24" s="6" t="s">
+      <c r="J24" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K24" s="6" t="s">
+      <c r="K24" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
-      <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
-      <c r="T24" s="6"/>
-      <c r="U24" s="6" t="s">
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="V24" s="6"/>
-      <c r="W24" s="6"/>
-      <c r="X24" s="6"/>
-      <c r="Y24" s="6"/>
-      <c r="Z24" s="6"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+      <c r="X24" s="5"/>
+      <c r="Y24" s="5"/>
+      <c r="Z24" s="5"/>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" t="s">
         <v>150</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="3" t="s">
+      <c r="B25" s="5"/>
+      <c r="C25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="2">
         <v>100</v>
       </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6" t="s">
+      <c r="G25" s="5"/>
+      <c r="H25" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="J25" s="6" t="s">
+      <c r="J25" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="K25" s="6" t="s">
+      <c r="K25" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
-      <c r="T25" s="6"/>
-      <c r="U25" s="6" t="s">
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="V25" s="6"/>
-      <c r="W25" s="6"/>
-      <c r="X25" s="6"/>
-      <c r="Y25" s="6"/>
-      <c r="Z25" s="6"/>
+      <c r="V25" s="5"/>
+      <c r="W25" s="5"/>
+      <c r="X25" s="5"/>
+      <c r="Y25" s="5"/>
+      <c r="Z25" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3143,19 +3807,19 @@
       <c r="I1" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>23</v>
       </c>
       <c r="O1" t="s">
@@ -3176,82 +3840,82 @@
       <c r="T1" t="s">
         <v>29</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>31</v>
       </c>
       <c r="W1" t="s">
         <v>32</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>100</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="5" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="N2" s="5"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="3" t="s">
+      <c r="N2" s="4"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6" t="s">
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="T2" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
-      <c r="Z2" s="3"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -3302,18 +3966,18 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>159</v>
       </c>
     </row>
@@ -3334,18 +3998,18 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>160</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated messaging module tc with admin validations
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="28"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="42"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -37,13 +37,25 @@
     <sheet name="OwnAccountTransferData" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="OtherAccountTransfersData" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="OtherCreditCardTransferData" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="MDraftMessageData" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="MBillPaymentDisputeData" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="MInboxAndRestoreData" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="MOtherSubjectValidationData" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="MFundTransferDisputeData" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="MBalanceConfirmationData" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="MFundTransferRequestData" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="MCardCenterValidationData" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="MFdInquiryAndSendMailData" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="LoginDataAlternateFour" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="SavingsAccountNumber" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="FDCompleteFlowData" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="346">
   <si>
     <t>userName</t>
   </si>
@@ -688,6 +700,9 @@
   </si>
   <si>
     <t>nickName</t>
+  </si>
+  <si>
+    <t>1000.00</t>
   </si>
   <si>
     <t>TestUser100</t>
@@ -854,13 +869,238 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>successMsg</t>
+  </si>
+  <si>
+    <t>otp</t>
+  </si>
+  <si>
+    <t>messageCreationSuccessMsg</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t>updatedMsg</t>
+  </si>
+  <si>
+    <t>deletionSuccessMsg</t>
+  </si>
+  <si>
+    <t>filePath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill Payment Dispute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Created New Message Thread Successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto DM message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">updated message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message Deleted Successfully!</t>
+  </si>
+  <si>
+    <t>12752-transaction.pdf</t>
+  </si>
+  <si>
+    <t>headerTile</t>
+  </si>
+  <si>
+    <t>1111111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUto BPD message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login to Vishwa Retail Admin</t>
+  </si>
+  <si>
+    <t>udarasom</t>
+  </si>
+  <si>
+    <t>abc@1234</t>
+  </si>
+  <si>
+    <t>responseMsg</t>
+  </si>
+  <si>
+    <t>messageDeletionSuccessMsg</t>
+  </si>
+  <si>
+    <t>messageRecoverySuccessMsg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fund Transfer Dispute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto IR message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message Recovered Successfully!</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto OS message</t>
+  </si>
+  <si>
+    <t>Hikkaduwa</t>
+  </si>
+  <si>
+    <t>kolithal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto FTD message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance Confirmation Request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto BCR message</t>
+  </si>
+  <si>
+    <t>nipunar</t>
+  </si>
+  <si>
+    <t>accountNo</t>
+  </si>
+  <si>
+    <t>remark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fund Transfer Request</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>111111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto FTR message</t>
+  </si>
+  <si>
+    <t>199812345678</t>
+  </si>
+  <si>
+    <t>RemarkAuto</t>
+  </si>
+  <si>
+    <t>subCategory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto Card C message 1</t>
+  </si>
+  <si>
+    <t>nimanthar</t>
+  </si>
+  <si>
+    <t>forwardMessage</t>
+  </si>
+  <si>
+    <t>branchUserName</t>
+  </si>
+  <si>
+    <t>branchPassword</t>
+  </si>
+  <si>
+    <t>CBOUUserName</t>
+  </si>
+  <si>
+    <t>CBOUPassword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed Deposit Inquiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation test message 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forward message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMS sent successfully to the registered mobile number:******9261</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>rate</t>
+  </si>
+  <si>
+    <t>interest</t>
+  </si>
+  <si>
+    <t>totalAmount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoax@1234 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sampath Sanhinda Fixed Deposit</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6  Months</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8.00</t>
+  </si>
+  <si>
+    <t>100000.00</t>
+  </si>
+  <si>
+    <t>fahimmohamed </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sampath Fixed Deposit</t>
+  </si>
+  <si>
+    <t>106250061318</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1  Months </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.00 </t>
+  </si>
+  <si>
+    <t>25000.00</t>
+  </si>
+  <si>
+    <t>238.36</t>
+  </si>
+  <si>
+    <t>25238.36</t>
+  </si>
+  <si>
+    <t>TestUser101</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -897,6 +1137,20 @@
       <color rgb="FF067D17"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10.000000"/>
+      <color rgb="FF7A7E85"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF6AAB73"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -918,7 +1172,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
@@ -959,9 +1213,8 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="4" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -971,18 +1224,33 @@
     <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="9" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2160,11 +2428,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1000</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" s="15" t="s">
         <v>215</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2198,7 +2466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -2230,7 +2498,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -2257,22 +2525,22 @@
   <sheetData>
     <row r="1" ht="57">
       <c r="A1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>197</v>
@@ -2283,19 +2551,19 @@
       <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="15" t="s">
-        <v>224</v>
+      <c r="J1" s="4" t="s">
+        <v>225</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" ht="85.5">
       <c r="A2" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C2" s="5">
         <v>14</v>
@@ -2304,25 +2572,25 @@
         <v>50001</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="H2" s="16" t="s">
         <v>231</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>232</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="17">
+      <c r="J2" s="18">
         <v>0</v>
       </c>
-      <c r="K2" s="17" t="s">
-        <v>232</v>
+      <c r="K2" s="18" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -2384,19 +2652,19 @@
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F1" t="s">
         <v>197</v>
@@ -2408,21 +2676,21 @@
         <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J1" t="s">
         <v>29</v>
       </c>
       <c r="K1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" ht="42.75">
       <c r="A2" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2431,28 +2699,28 @@
         <v>50001</v>
       </c>
       <c r="D2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="G2" s="19" t="s">
-        <v>231</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>39</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L2" s="5">
         <v>2</v>
@@ -2476,43 +2744,43 @@
   <sheetData>
     <row r="1" s="4" customFormat="1" ht="57">
       <c r="A1" s="20" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>29</v>
@@ -2521,81 +2789,676 @@
         <v>13</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" s="4" customFormat="1" ht="114">
-      <c r="A2" s="22" t="s">
-        <v>258</v>
-      </c>
-      <c r="B2" s="22" t="s">
+      <c r="A2" s="18" t="s">
         <v>259</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="B2" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="C2" s="18" t="s">
         <v>261</v>
       </c>
-      <c r="E2" s="22" t="s">
-        <v>227</v>
-      </c>
-      <c r="F2" s="22" t="s">
+      <c r="D2" s="18" t="s">
         <v>262</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="E2" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>263</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="G2" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="I2" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="J2" s="22" t="s">
+      <c r="H2" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="I2" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="J2" s="18" t="s">
         <v>266</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="K2" s="18" t="s">
         <v>267</v>
       </c>
-      <c r="M2" s="22">
+      <c r="L2" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="M2" s="18">
         <v>30001</v>
       </c>
-      <c r="N2" s="22" t="s">
-        <v>242</v>
-      </c>
-      <c r="O2" s="22" t="s">
+      <c r="N2" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="O2" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="P2" s="22" t="s">
-        <v>268</v>
-      </c>
-      <c r="Q2" s="22">
+      <c r="P2" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q2" s="18">
         <v>501</v>
       </c>
-      <c r="R2" s="22">
+      <c r="R2" s="18">
         <v>0</v>
       </c>
-      <c r="S2" s="23" t="s">
-        <v>269</v>
-      </c>
-      <c r="T2" s="23" t="s">
-        <v>232</v>
+      <c r="S2" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="T2" s="18" t="s">
+        <v>233</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="17.57421875"/>
+    <col customWidth="1" min="4" max="4" width="27.00390625"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>276</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="16">
+        <v>1111111</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>284</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" ht="14.25">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G1" t="s">
+        <v>285</v>
+      </c>
+      <c r="H1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>287</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>291</v>
+      </c>
+      <c r="G1" t="s">
+        <v>292</v>
+      </c>
+      <c r="H1" t="s">
+        <v>293</v>
+      </c>
+      <c r="I1" t="s">
+        <v>285</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="s">
+        <v>294</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>295</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="L2" s="16" t="s">
+        <v>284</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>285</v>
+      </c>
+      <c r="G1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="s">
+        <v>294</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>284</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>285</v>
+      </c>
+      <c r="G1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="5" max="5" width="20.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D1" t="s">
+        <v>273</v>
+      </c>
+      <c r="E1" t="s">
+        <v>274</v>
+      </c>
+      <c r="F1" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H1" t="s">
+        <v>307</v>
+      </c>
+      <c r="I1" t="s">
+        <v>285</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="s">
+        <v>308</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>311</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="17.7109375"/>
+    <col customWidth="1" min="5" max="5" width="18.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D1" t="s">
+        <v>273</v>
+      </c>
+      <c r="E1" t="s">
+        <v>274</v>
+      </c>
+      <c r="F1" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" t="s">
+        <v>285</v>
+      </c>
+      <c r="H1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="16">
+        <v>111111</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2633,6 +3496,280 @@
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="5" max="5" width="30.140625"/>
+    <col customWidth="1" min="7" max="7" width="19.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D1" t="s">
+        <v>273</v>
+      </c>
+      <c r="E1" t="s">
+        <v>274</v>
+      </c>
+      <c r="F1" t="s">
+        <v>275</v>
+      </c>
+      <c r="G1" t="s">
+        <v>318</v>
+      </c>
+      <c r="H1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1" t="s">
+        <v>319</v>
+      </c>
+      <c r="J1" t="s">
+        <v>320</v>
+      </c>
+      <c r="K1" t="s">
+        <v>321</v>
+      </c>
+      <c r="L1" t="s">
+        <v>322</v>
+      </c>
+      <c r="M1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="M2" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>326</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="21.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
+        <v>218</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>326</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>334</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="I2" s="16">
+        <v>3989.04</v>
+      </c>
+      <c r="J2" s="16">
+        <v>103989.03999999999</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" ht="71.25">
+      <c r="A3" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>338</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>339</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated messaging module and reporter module
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="42"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="40"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -46,16 +46,17 @@
     <sheet name="MFundTransferRequestData" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="MCardCenterValidationData" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="MFdInquiryAndSendMailData" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="LoginDataAlternateFour" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="SavingsAccountNumber" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="FDCompleteFlowData" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="MComposeNewMessageData" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="LoginDataAlternateFour" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="SavingsAccountNumber" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="FDCompleteFlowData" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="364">
   <si>
     <t>userName</t>
   </si>
@@ -576,7 +577,7 @@
     <t xml:space="preserve">1001 5102 6073</t>
   </si>
   <si>
-    <t xml:space="preserve">LKR 8,530.00</t>
+    <t xml:space="preserve">LKR 8,505.00</t>
   </si>
   <si>
     <t xml:space="preserve">DOUBLE S SAVINGS -PERSONAL</t>
@@ -1034,6 +1035,61 @@
   </si>
   <si>
     <t xml:space="preserve">Forward message</t>
+  </si>
+  <si>
+    <t>uploadErrorMsg</t>
+  </si>
+  <si>
+    <t>fileNameOne</t>
+  </si>
+  <si>
+    <t>fileNameTwo</t>
+  </si>
+  <si>
+    <t>fileNameThree</t>
+  </si>
+  <si>
+    <t>fileNameFour</t>
+  </si>
+  <si>
+    <t>fileNameFive</t>
+  </si>
+  <si>
+    <t>pastedText</t>
+  </si>
+  <si>
+    <t>sanitizedExpected</t>
+  </si>
+  <si>
+    <t>testInputWithSpecialCharacters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exceeds the maximum size of 512KB</t>
+  </si>
+  <si>
+    <t>Message_JPEG.JPEG</t>
+  </si>
+  <si>
+    <t>Message_JPG.JPG</t>
+  </si>
+  <si>
+    <t>Message_PNG.PNG</t>
+  </si>
+  <si>
+    <t>Message_PDF.PDF</t>
+  </si>
+  <si>
+    <t>Message_PDF_1MB.PDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> This is   a 
+ test    message  with   spacing and alignment.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a test message with spacing and alignment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">123ABCabc!@#$%^&amp;*()_+-=[]{}|;':",.&lt;&gt;?/ </t>
   </si>
   <si>
     <t xml:space="preserve">SMS sent successfully to the registered mobile number:******9261</t>
@@ -1172,7 +1228,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="26">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
@@ -1213,8 +1269,6 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="4" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1230,7 +1284,6 @@
     <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="7" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1240,12 +1293,7 @@
     <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="9" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -2428,10 +2476,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="5" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2580,16 +2628,16 @@
       <c r="G2" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="15" t="s">
         <v>232</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="18">
+      <c r="J2" s="16">
         <v>0</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="16" t="s">
         <v>233</v>
       </c>
     </row>
@@ -2701,7 +2749,7 @@
       <c r="D2" t="s">
         <v>233</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="17" t="s">
         <v>230</v>
       </c>
       <c r="F2" s="5" t="s">
@@ -2743,10 +2791,10 @@
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1" ht="57">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="19" t="s">
         <v>246</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -2770,7 +2818,7 @@
       <c r="I1" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="19" t="s">
         <v>254</v>
       </c>
       <c r="K1" s="4" t="s">
@@ -2805,64 +2853,64 @@
       </c>
     </row>
     <row r="2" s="4" customFormat="1" ht="114">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="16" t="s">
         <v>260</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="16" t="s">
         <v>261</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="16" t="s">
         <v>262</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="16" t="s">
         <v>263</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="16" t="s">
         <v>264</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="16" t="s">
         <v>266</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="16" t="s">
         <v>267</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="16" t="s">
         <v>268</v>
       </c>
-      <c r="M2" s="18">
+      <c r="M2" s="16">
         <v>30001</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="N2" s="16" t="s">
         <v>243</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="O2" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="16" t="s">
         <v>269</v>
       </c>
-      <c r="Q2" s="18">
+      <c r="Q2" s="16">
         <v>501</v>
       </c>
-      <c r="R2" s="18">
+      <c r="R2" s="16">
         <v>0</v>
       </c>
-      <c r="S2" s="18" t="s">
+      <c r="S2" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="T2" s="18" t="s">
+      <c r="T2" s="16" t="s">
         <v>233</v>
       </c>
     </row>
@@ -2880,6 +2928,7 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="17.57421875"/>
     <col customWidth="1" min="4" max="4" width="27.00390625"/>
+    <col customWidth="1" min="8" max="8" width="20.57421875"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -2901,36 +2950,36 @@
       <c r="F1" t="s">
         <v>276</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="3" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="16">
+      <c r="C2" s="5">
         <v>1111111</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="5" t="s">
         <v>284</v>
       </c>
     </row>
@@ -2976,31 +3025,31 @@
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>290</v>
       </c>
     </row>
@@ -3014,10 +3063,10 @@
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="3" t="s">
         <v>271</v>
       </c>
       <c r="B1" t="s">
@@ -3055,40 +3104,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="5" t="s">
         <v>284</v>
       </c>
     </row>
@@ -3102,10 +3151,10 @@
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="21" t="s">
         <v>271</v>
       </c>
       <c r="B1" t="s">
@@ -3137,34 +3186,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="5" t="s">
         <v>290</v>
       </c>
     </row>
@@ -3178,7 +3227,7 @@
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -3210,31 +3259,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>284</v>
       </c>
     </row>
@@ -3248,7 +3297,7 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -3277,28 +3326,28 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>290</v>
       </c>
     </row>
@@ -3312,13 +3361,13 @@
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="5" max="5" width="20.28125"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="21" t="s">
         <v>271</v>
       </c>
       <c r="B1" t="s">
@@ -3353,37 +3402,37 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="5" t="s">
         <v>290</v>
       </c>
     </row>
@@ -3397,7 +3446,7 @@
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="3" max="3" width="17.7109375"/>
     <col customWidth="1" min="5" max="5" width="18.8515625"/>
@@ -3433,31 +3482,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="5">
         <v>111111</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="5" t="s">
         <v>290</v>
       </c>
     </row>
@@ -3508,7 +3557,7 @@
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="5" max="5" width="30.140625"/>
     <col customWidth="1" min="7" max="7" width="19.57421875"/>
@@ -3559,40 +3608,40 @@
       <c r="A2" t="s">
         <v>323</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="22" t="s">
         <v>300</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="L2" s="15" t="s">
+      <c r="L2" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -3606,28 +3655,80 @@
 
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="33.57421875"/>
+    <col customWidth="1" min="2" max="2" width="36.140625"/>
+    <col customWidth="1" min="3" max="3" width="14.140625"/>
+    <col customWidth="1" min="6" max="6" width="18.140625"/>
+    <col customWidth="1" min="7" max="7" width="31.7109375"/>
+    <col customWidth="1" min="8" max="8" width="43.8515625"/>
+    <col customWidth="1" min="9" max="9" width="40.28125"/>
+    <col customWidth="1" min="10" max="10" width="58.7109375"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="26" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="26" t="s">
-        <v>217</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="26" t="s">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
         <v>326</v>
+      </c>
+      <c r="C1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D1" t="s">
+        <v>328</v>
+      </c>
+      <c r="E1" t="s">
+        <v>329</v>
+      </c>
+      <c r="F1" t="s">
+        <v>330</v>
+      </c>
+      <c r="G1" t="s">
+        <v>331</v>
+      </c>
+      <c r="H1" t="s">
+        <v>332</v>
+      </c>
+      <c r="I1" t="s">
+        <v>333</v>
+      </c>
+      <c r="J1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" ht="42.75">
+      <c r="A2" s="23" t="s">
+        <v>294</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="H2" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -3640,19 +3741,28 @@
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="21.57421875"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>17</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
-        <v>218</v>
+      <c r="A2" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -3665,10 +3775,35 @@
 
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="21.57421875"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -3678,98 +3813,98 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>332</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>326</v>
+      <c r="B2" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>344</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="E2" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>334</v>
-      </c>
-      <c r="G2" s="16" t="s">
-        <v>335</v>
-      </c>
-      <c r="H2" s="16" t="s">
-        <v>336</v>
-      </c>
-      <c r="I2" s="16">
+      <c r="F2" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="I2" s="5">
         <v>3989.04</v>
       </c>
-      <c r="J2" s="16">
+      <c r="J2" s="5">
         <v>103989.03999999999</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="5" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="3" ht="71.25">
-      <c r="A3" s="16" t="s">
-        <v>337</v>
+      <c r="A3" s="5" t="s">
+        <v>355</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="C3" s="28" t="s">
+        <v>350</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="29" t="s">
-        <v>338</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>339</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>340</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>341</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>342</v>
-      </c>
-      <c r="I3" s="16" t="s">
-        <v>343</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>344</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>345</v>
+      <c r="D3" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added My account and modules under my account with minor enhancements in other modules that impact My account
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="40"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="50"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -48,15 +48,22 @@
     <sheet name="MFdInquiryAndSendMailData" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="MComposeNewMessageData" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="LoginDataAlternateFour" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="SavingsAccountNumber" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="FDCompleteFlowData" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="LoginDataAlternateFive" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="SavingsAccountNumber" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="FDCompleteFlowData" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="PawningData" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="LoanDetails" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="SADetailedViewData" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="CADetailedViewData" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="ChequeRequestData" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="AdvancedSearchData" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="405">
   <si>
     <t>userName</t>
   </si>
@@ -782,7 +789,7 @@
 Insufficient funds in the selected account</t>
   </si>
   <si>
-    <t>2550040541</t>
+    <t>002550040541</t>
   </si>
   <si>
     <t>Baabu</t>
@@ -1150,6 +1157,129 @@
   </si>
   <si>
     <t>TestUser101</t>
+  </si>
+  <si>
+    <t>minimumAmount</t>
+  </si>
+  <si>
+    <t>maximumAmount</t>
+  </si>
+  <si>
+    <t>actualAmount</t>
+  </si>
+  <si>
+    <t>wrongMonth</t>
+  </si>
+  <si>
+    <t>correctMonth</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>500000</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing the obtain loan</t>
+  </si>
+  <si>
+    <t>accHolderName</t>
+  </si>
+  <si>
+    <t>systemReserved</t>
+  </si>
+  <si>
+    <t>lienAmount</t>
+  </si>
+  <si>
+    <t>accOpenedOn</t>
+  </si>
+  <si>
+    <t>accountBalance</t>
+  </si>
+  <si>
+    <t>floatBalance</t>
+  </si>
+  <si>
+    <t>amountFrom</t>
+  </si>
+  <si>
+    <t>amountTo</t>
+  </si>
+  <si>
+    <t>102555130162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUST NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 27,000.00</t>
+  </si>
+  <si>
+    <t>21-07-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 2,116.00</t>
+  </si>
+  <si>
+    <t>123.00</t>
+  </si>
+  <si>
+    <t>odLimit</t>
+  </si>
+  <si>
+    <t>tempOdLimit</t>
+  </si>
+  <si>
+    <t>overdueLiability</t>
+  </si>
+  <si>
+    <t>reservedAmount</t>
+  </si>
+  <si>
+    <t>openedOn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 150,000.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 230,870.86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR 53,776.17</t>
+  </si>
+  <si>
+    <t>18-02-2020</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>from</t>
+  </si>
+  <si>
+    <t>to</t>
+  </si>
+  <si>
+    <t>fullDate</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>5.00</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1358,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
@@ -1293,12 +1423,19 @@
     <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="9" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3700,7 +3837,7 @@
       </c>
     </row>
     <row r="2" ht="42.75">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="5" t="s">
         <v>294</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -3777,17 +3914,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.57421875"/>
+    <col customWidth="1" min="1" max="1" width="24.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>17</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>218</v>
+      <c r="A2" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3801,6 +3950,31 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="21.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
@@ -3879,10 +4053,10 @@
       <c r="B3" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="24" t="s">
         <v>356</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -3905,6 +4079,263 @@
       </c>
       <c r="K3" s="5" t="s">
         <v>363</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>372</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="5" style="25" width="9.140625"/>
+    <col customWidth="1" min="6" max="6" style="25" width="38.421875"/>
+    <col min="7" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>372</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col bestFit="1" min="1" max="1" style="25" width="14.57421875"/>
+    <col bestFit="1" min="2" max="2" style="25" width="14.140625"/>
+    <col bestFit="1" min="3" max="3" style="25" width="14.7109375"/>
+    <col bestFit="1" min="4" max="4" style="25" width="10.7109375"/>
+    <col bestFit="1" min="5" max="5" style="25" width="12.8515625"/>
+    <col bestFit="1" min="6" max="6" style="25" width="14.140625"/>
+    <col bestFit="1" min="7" max="7" style="25" width="11.140625"/>
+    <col bestFit="1" min="8" max="8" style="25" width="12.140625"/>
+    <col min="9" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>374</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>375</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>376</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>377</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>378</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>379</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>380</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="s">
+        <v>382</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>383</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>385</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>386</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>387</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>388</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>388</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="5" style="25" width="9.140625"/>
+    <col bestFit="1" min="6" max="6" style="25" width="14.140625"/>
+    <col bestFit="1" min="7" max="7" style="25" width="9.8515625"/>
+    <col min="8" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>389</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>391</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>392</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>378</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>394</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>395</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>396</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -5024,6 +5455,98 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="Z23"/>
   </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="16384" style="25" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>346</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>398</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>399</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>400</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>401</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>380</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>402</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>403</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>403</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>386</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>404</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>404</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>

<commit_message>
Mild changes to Data provider and data sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="50"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="46"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -59,11 +59,14 @@
     <sheet name="AdvancedSearchData" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="409">
   <si>
     <t>userName</t>
   </si>
@@ -1187,6 +1190,18 @@
   </si>
   <si>
     <t xml:space="preserve">Testing the obtain loan</t>
+  </si>
+  <si>
+    <t>accountNumber1</t>
+  </si>
+  <si>
+    <t>accountNumber2</t>
+  </si>
+  <si>
+    <t>216758079687</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0167 5100 0165</t>
   </si>
   <si>
     <t>accHolderName</t>
@@ -1358,7 +1373,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
@@ -1429,7 +1444,6 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -4093,11 +4107,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" style="25" width="9.140625"/>
+    <col min="1" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="25" t="s">
         <v>364</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -4117,22 +4131,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="5" t="s">
         <v>373</v>
       </c>
     </row>
@@ -4146,51 +4160,64 @@
 
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="5" style="25" width="9.140625"/>
-    <col customWidth="1" min="6" max="6" style="25" width="38.421875"/>
-    <col min="7" max="16384" style="25" width="9.140625"/>
+    <col min="1" max="1" style="5" width="9.140625"/>
+    <col min="2" max="6" style="5" width="9.140625"/>
+    <col customWidth="1" min="7" max="7" style="5" width="38.421875"/>
+    <col min="8" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>364</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="H1" s="26" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
+        <v>376</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="C2" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="E2" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F2" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="G2" s="5" t="s">
         <v>373</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -4205,73 +4232,73 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col bestFit="1" min="1" max="1" style="25" width="14.57421875"/>
-    <col bestFit="1" min="2" max="2" style="25" width="14.140625"/>
-    <col bestFit="1" min="3" max="3" style="25" width="14.7109375"/>
-    <col bestFit="1" min="4" max="4" style="25" width="10.7109375"/>
-    <col bestFit="1" min="5" max="5" style="25" width="12.8515625"/>
-    <col bestFit="1" min="6" max="6" style="25" width="14.140625"/>
-    <col bestFit="1" min="7" max="7" style="25" width="11.140625"/>
-    <col bestFit="1" min="8" max="8" style="25" width="12.140625"/>
-    <col min="9" max="16384" style="25" width="9.140625"/>
+    <col bestFit="1" min="1" max="1" style="5" width="14.57421875"/>
+    <col bestFit="1" min="2" max="2" style="5" width="14.140625"/>
+    <col bestFit="1" min="3" max="3" style="5" width="14.7109375"/>
+    <col bestFit="1" min="4" max="4" style="5" width="10.7109375"/>
+    <col bestFit="1" min="5" max="5" style="5" width="12.8515625"/>
+    <col bestFit="1" min="6" max="6" style="5" width="14.140625"/>
+    <col bestFit="1" min="7" max="7" style="5" width="11.140625"/>
+    <col bestFit="1" min="8" max="8" style="5" width="12.140625"/>
+    <col min="9" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>374</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>375</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>376</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>377</v>
-      </c>
-      <c r="F1" s="27" t="s">
+      <c r="B1" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="C1" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="D1" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="E1" s="5" t="s">
         <v>381</v>
       </c>
+      <c r="F1" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>385</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="s">
-        <v>382</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>383</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>384</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>385</v>
-      </c>
-      <c r="E2" s="27" t="s">
+      <c r="A2" s="5" t="s">
         <v>386</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="B2" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="G2" s="27" t="s">
-        <v>384</v>
-      </c>
-      <c r="H2" s="28" t="s">
+      <c r="C2" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="I2" s="27" t="s">
+      <c r="D2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>388</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>392</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -4286,56 +4313,56 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="5" style="25" width="9.140625"/>
-    <col bestFit="1" min="6" max="6" style="25" width="14.140625"/>
-    <col bestFit="1" min="7" max="7" style="25" width="9.8515625"/>
-    <col min="8" max="16384" style="25" width="9.140625"/>
+    <col min="1" max="5" style="5" width="9.140625"/>
+    <col bestFit="1" min="6" max="6" style="5" width="14.140625"/>
+    <col bestFit="1" min="7" max="7" style="5" width="9.8515625"/>
+    <col min="8" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>389</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>390</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>391</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>392</v>
-      </c>
-      <c r="F1" s="27" t="s">
-        <v>378</v>
-      </c>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="5" t="s">
         <v>393</v>
       </c>
+      <c r="C1" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>397</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>394</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>384</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>395</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>384</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>396</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>397</v>
+      <c r="B2" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -5466,16 +5493,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" style="25" width="9.140625"/>
+    <col min="1" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>241</v>
       </c>
     </row>
@@ -5489,62 +5516,67 @@
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" style="25" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" style="5" width="18.8515625"/>
+    <col min="2" max="16384" style="5" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="C1" s="27" t="s">
-        <v>398</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>399</v>
-      </c>
-      <c r="E1" s="27" t="s">
-        <v>400</v>
-      </c>
-      <c r="F1" s="27" t="s">
-        <v>401</v>
-      </c>
-      <c r="G1" s="27" t="s">
-        <v>380</v>
-      </c>
-      <c r="H1" s="27" t="s">
-        <v>381</v>
-      </c>
+      <c r="C1" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>402</v>
-      </c>
-      <c r="C2" s="27" t="s">
+      <c r="B2" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D2" s="27" t="s">
-        <v>403</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>403</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>386</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>404</v>
-      </c>
-      <c r="H2" s="27" t="s">
-        <v>404</v>
-      </c>
+      <c r="D2" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>